<commit_message>
-Se amplio el analisis con gráficos de los resultados obtenidos en la medicion de tiempos y del uso de la memoria y cpu
</commit_message>
<xml_diff>
--- a/metricas_realizadas/SOA/Analisis Metricas SOA/Resultados Medicion Tiempos desarrollo.xlsx
+++ b/metricas_realizadas/SOA/Analisis Metricas SOA/Resultados Medicion Tiempos desarrollo.xlsx
@@ -8,15 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyecto_code_ia\metricas_realizadas\SOA\Analisis Metricas SOA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD283BD6-3A68-492B-B461-0C9A1B26ADB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F0AD829-432E-4F26-B46F-85210C215A75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tiempos ESP32" sheetId="1" r:id="rId1"/>
     <sheet name="Tiempos Android" sheetId="2" r:id="rId2"/>
-    <sheet name="Analisis de tiempos" sheetId="4" r:id="rId3"/>
+    <sheet name="Analisis de tiempos ESP32" sheetId="4" r:id="rId3"/>
+    <sheet name="Analisis tiempo Android" sheetId="5" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">'Tiempos ESP32'!$J$27</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">'Tiempos ESP32'!$A$24</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">'Tiempos ESP32'!$A$24:$A$30</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">'Tiempos ESP32'!$A$25:$A$30</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">'Tiempos ESP32'!$D$24:$D$30</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">'Tiempos ESP32'!$D$25:$D$30</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">'Tiempos ESP32'!$J$27</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="40">
   <si>
     <t>Grupo</t>
   </si>
@@ -137,6 +147,30 @@
   <si>
     <t>HORAS DE DESARROLLO IA  EN ESP32</t>
   </si>
+  <si>
+    <t>DATOS ESTADISTICOS</t>
+  </si>
+  <si>
+    <t>Manual</t>
+  </si>
+  <si>
+    <t>IA</t>
+  </si>
+  <si>
+    <t>Speedup</t>
+  </si>
+  <si>
+    <t>Reducción</t>
+  </si>
+  <si>
+    <t>PORCENTAJE DE REDUCCION DE TIEMPO</t>
+  </si>
+  <si>
+    <t>Promedio IA</t>
+  </si>
+  <si>
+    <t>Speedup promedio</t>
+  </si>
 </sst>
 </file>
 
@@ -173,7 +207,7 @@
       <name val="Roboto"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -204,8 +238,38 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF356854"/>
+        <bgColor rgb="FF356854"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7030A0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -243,11 +307,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF356854"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF356854"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF356854"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -278,6 +362,36 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1259,6 +1373,2141 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-AR"/>
+              <a:t>Porcentaje</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-AR" baseline="0"/>
+              <a:t> de reducción de tiempo al usar IA </a:t>
+            </a:r>
+          </a:p>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-AR" baseline="0"/>
+              <a:t>con respecto del desarrollo manual</a:t>
+            </a:r>
+            <a:endParaRPr lang="es-AR"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-AR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Tiempos ESP32'!$A$34</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>L1</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="es-AR"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Tiempos ESP32'!$B$33</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Reducción</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Tiempos ESP32'!$B$34</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>92.982456140350877</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-DD80-4AF1-9B96-D31528765867}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Tiempos ESP32'!$A$35</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>L2</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="es-AR"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Tiempos ESP32'!$B$33</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Reducción</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Tiempos ESP32'!$B$35</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>80</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-DD80-4AF1-9B96-D31528765867}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Tiempos ESP32'!$A$36</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>M1</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent3"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="es-AR"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Tiempos ESP32'!$B$33</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Reducción</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Tiempos ESP32'!$B$36</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>85.365853658536579</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-DD80-4AF1-9B96-D31528765867}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Tiempos ESP32'!$A$37</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>M2</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent4"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="es-AR"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Tiempos ESP32'!$B$33</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Reducción</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Tiempos ESP32'!$B$37</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>91.428571428571431</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-DD80-4AF1-9B96-D31528765867}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Tiempos ESP32'!$A$38</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>M4</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent5"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="es-AR"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Tiempos ESP32'!$B$33</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Reducción</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Tiempos ESP32'!$B$38</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>82.758620689655174</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-DD80-4AF1-9B96-D31528765867}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Tiempos ESP32'!$A$39</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>M5</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent6"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="es-AR"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Tiempos ESP32'!$B$33</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Reducción</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Tiempos ESP32'!$B$39</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>72.727272727272734</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000005-DD80-4AF1-9B96-D31528765867}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1260099120"/>
+        <c:axId val="1260100368"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1260099120"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="es-AR"/>
+                  <a:t>Grupos</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="es-AR"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1260100368"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1260100368"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="es-AR"/>
+                  <a:t>Porcentaje</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="es-AR"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-AR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1260099120"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-AR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-AR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-AR"/>
+              <a:t>Desarrollo</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-AR" baseline="0"/>
+              <a:t> ESP32 Manual Vs IA</a:t>
+            </a:r>
+            <a:endParaRPr lang="es-AR"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-AR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Tiempos ESP32'!$B$24</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Manual</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Tiempos ESP32'!$A$25:$A$30</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>L1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>L2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>M1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>M2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>M4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>M5</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Tiempos ESP32'!$B$25:$B$30</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>28.5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>22</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-9DFF-499B-975D-9E1F357E1424}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Tiempos ESP32'!$C$24</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>IA</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Tiempos ESP32'!$A$25:$A$30</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>L1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>L2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>M1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>M2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>M4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>M5</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Tiempos ESP32'!$C$25:$C$30</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-9DFF-499B-975D-9E1F357E1424}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1147789600"/>
+        <c:axId val="1147792928"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1147789600"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="es-AR"/>
+                  <a:t>Grupos</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="es-AR"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-AR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1147792928"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1147792928"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="es-AR"/>
+                  <a:t>Cant.</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="es-AR" baseline="0"/>
+                  <a:t>  de horas</a:t>
+                </a:r>
+                <a:endParaRPr lang="es-AR"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="es-AR"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-AR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1147789600"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-AR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-AR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-AR"/>
+              <a:t>Speedup ESP32 Manual</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-AR" baseline="0"/>
+              <a:t> vs IA</a:t>
+            </a:r>
+            <a:endParaRPr lang="es-AR"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-AR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Tiempos ESP32'!$D$24</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Speedup</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-F174-494B-B444-83599EA18FD9}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-F174-494B-B444-83599EA18FD9}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-F174-494B-B444-83599EA18FD9}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-F174-494B-B444-83599EA18FD9}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000009-F174-494B-B444-83599EA18FD9}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="5"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000B-F174-494B-B444-83599EA18FD9}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="es-AR"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>('Tiempos ESP32'!$A$25,'Tiempos ESP32'!$A$26,'Tiempos ESP32'!$A$27,'Tiempos ESP32'!$A$28,'Tiempos ESP32'!$A$29,'Tiempos ESP32'!$A$30)</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>L1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>L2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>M1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>M2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>M4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>M5</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>('Tiempos ESP32'!$D$25,'Tiempos ESP32'!$D$26,'Tiempos ESP32'!$D$27,'Tiempos ESP32'!$D$28,'Tiempos ESP32'!$D$29,'Tiempos ESP32'!$D$30)</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>14.25</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6.833333333333333</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>11.666666666666666</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5.8</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3.6666666666666665</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000C-F174-494B-B444-83599EA18FD9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:axId val="1146753568"/>
+        <c:axId val="1146754816"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1146753568"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-AR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1146754816"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1146754816"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-AR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1146753568"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-AR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-AR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
               <a:defRPr sz="1800" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="dk1">
@@ -1368,7 +3617,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-3172-4033-8972-83ACD8272B6B}"/>
+                <c16:uniqueId val="{00000001-B73A-421D-999E-0569B5DA5F0C}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1393,7 +3642,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000003-3172-4033-8972-83ACD8272B6B}"/>
+                <c16:uniqueId val="{00000003-B73A-421D-999E-0569B5DA5F0C}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1418,7 +3667,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000005-3172-4033-8972-83ACD8272B6B}"/>
+                <c16:uniqueId val="{00000005-B73A-421D-999E-0569B5DA5F0C}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1443,7 +3692,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000007-3172-4033-8972-83ACD8272B6B}"/>
+                <c16:uniqueId val="{00000007-B73A-421D-999E-0569B5DA5F0C}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1468,7 +3717,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000009-3172-4033-8972-83ACD8272B6B}"/>
+                <c16:uniqueId val="{00000009-B73A-421D-999E-0569B5DA5F0C}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1493,7 +3742,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{0000000B-3172-4033-8972-83ACD8272B6B}"/>
+                <c16:uniqueId val="{0000000B-B73A-421D-999E-0569B5DA5F0C}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1509,7 +3758,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000001-3172-4033-8972-83ACD8272B6B}"/>
+                  <c16:uniqueId val="{00000001-B73A-421D-999E-0569B5DA5F0C}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -1524,7 +3773,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000003-3172-4033-8972-83ACD8272B6B}"/>
+                  <c16:uniqueId val="{00000003-B73A-421D-999E-0569B5DA5F0C}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -1539,7 +3788,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000005-3172-4033-8972-83ACD8272B6B}"/>
+                  <c16:uniqueId val="{00000005-B73A-421D-999E-0569B5DA5F0C}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -1554,7 +3803,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000007-3172-4033-8972-83ACD8272B6B}"/>
+                  <c16:uniqueId val="{00000007-B73A-421D-999E-0569B5DA5F0C}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -1569,7 +3818,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000009-3172-4033-8972-83ACD8272B6B}"/>
+                  <c16:uniqueId val="{00000009-B73A-421D-999E-0569B5DA5F0C}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -1584,7 +3833,7 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{0000000B-3172-4033-8972-83ACD8272B6B}"/>
+                  <c16:uniqueId val="{0000000B-B73A-421D-999E-0569B5DA5F0C}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -1713,7 +3962,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000C-3172-4033-8972-83ACD8272B6B}"/>
+              <c16:uniqueId val="{0000000C-B73A-421D-999E-0569B5DA5F0C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2147,6 +4396,126 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="253">
   <cs:axisTitle>
@@ -2749,6 +5118,1531 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="253">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -3391,23 +7285,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>50800</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>82550</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>31750</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="5" name="Gráfico 4">
+        <xdr:cNvPr id="7" name="Gráfico 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4A2918A5-EEF8-4510-ACC0-7074AFAB1B0F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8BBC83ED-51CC-4996-AA0F-5F168EE6F7FA}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3422,6 +7316,125 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>438150</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>438150</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>165100</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="8" name="Gráfico 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DE0C51C4-DDFC-402B-970E-C5C0C75F7581}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>527050</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>6350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>527050</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="9" name="Gráfico 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3E8E6710-E783-4A74-A00B-2F86D3A634E8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>165100</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Gráfico 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9F097900-DAAE-4B26-B7CF-08492423E0BC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3752,9 +7765,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="2" max="3" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="17.453125" customWidth="1"/>
     <col min="13" max="13" width="18.6328125" customWidth="1"/>
   </cols>
@@ -3818,7 +7832,7 @@
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="20" t="s">
         <v>12</v>
       </c>
       <c r="B3" s="3">
@@ -3857,7 +7871,7 @@
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="20" t="s">
         <v>13</v>
       </c>
       <c r="B4" s="3">
@@ -3896,7 +7910,7 @@
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="20" t="s">
         <v>14</v>
       </c>
       <c r="B5" s="3">
@@ -3938,7 +7952,7 @@
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="20" t="s">
         <v>15</v>
       </c>
       <c r="B6" s="3">
@@ -3980,7 +7994,7 @@
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B7" s="3">
@@ -4022,7 +8036,7 @@
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="20" t="s">
         <v>18</v>
       </c>
       <c r="B8" s="3">
@@ -4112,7 +8126,7 @@
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="20" t="s">
         <v>12</v>
       </c>
       <c r="B15" s="6">
@@ -4120,39 +8134,39 @@
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="20" t="s">
         <v>13</v>
       </c>
       <c r="B16" s="6">
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" s="3" t="s">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="B17" s="6">
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A18" s="3" t="s">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A18" s="20" t="s">
         <v>15</v>
       </c>
       <c r="B18" s="6">
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A19" s="3" t="s">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A19" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B19" s="6">
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A20" s="3" t="s">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A20" s="20" t="s">
         <v>18</v>
       </c>
       <c r="B20" s="6">
@@ -4162,19 +8176,287 @@
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" s="8"/>
       <c r="B21" s="11">
         <f>AVERAGE(B14:B20)</f>
         <v>4.5</v>
       </c>
     </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A23" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" s="18"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="18"/>
+      <c r="F23" s="18"/>
+      <c r="G23" s="18"/>
+      <c r="H23" s="18"/>
+      <c r="I23" s="18"/>
+      <c r="J23" s="18"/>
+      <c r="K23" s="18"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A24" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B24" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="C24" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="D24" s="19" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A25" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B25" s="17">
+        <f>M3</f>
+        <v>28.5</v>
+      </c>
+      <c r="C25" s="17">
+        <f>B15</f>
+        <v>2</v>
+      </c>
+      <c r="D25" s="23">
+        <f>B25/C25</f>
+        <v>14.25</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A26" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="B26" s="17">
+        <f t="shared" ref="B26:B30" si="0">M4</f>
+        <v>25</v>
+      </c>
+      <c r="C26" s="17">
+        <f t="shared" ref="C26:C30" si="1">B16</f>
+        <v>5</v>
+      </c>
+      <c r="D26" s="23">
+        <f t="shared" ref="D26:D30" si="2">B26/C26</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A27" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B27" s="17">
+        <f t="shared" si="0"/>
+        <v>41</v>
+      </c>
+      <c r="C27" s="17">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="D27" s="23">
+        <f t="shared" si="2"/>
+        <v>6.833333333333333</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A28" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="B28" s="17">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+      <c r="C28" s="17">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="D28" s="23">
+        <f t="shared" si="2"/>
+        <v>11.666666666666666</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A29" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="B29" s="17">
+        <f t="shared" si="0"/>
+        <v>29</v>
+      </c>
+      <c r="C29" s="17">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="D29" s="23">
+        <f t="shared" si="2"/>
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A30" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="B30" s="17">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="C30" s="17">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="D30" s="23">
+        <f t="shared" si="2"/>
+        <v>3.6666666666666665</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A31" s="22"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A32" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="B32" s="24"/>
+      <c r="C32" s="24"/>
+      <c r="D32" s="24"/>
+      <c r="E32" s="24"/>
+      <c r="F32" s="24"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B33" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="C33" s="19" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B34" s="26">
+        <f>((B25-C25)/B25)*100</f>
+        <v>92.982456140350877</v>
+      </c>
+      <c r="C34" s="23">
+        <f>D25</f>
+        <v>14.25</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="B35" s="26">
+        <f t="shared" ref="B35:B39" si="3">((B26-C26)/B26)*100</f>
+        <v>80</v>
+      </c>
+      <c r="C35" s="23">
+        <f t="shared" ref="C35:C39" si="4">D26</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B36" s="26">
+        <f t="shared" si="3"/>
+        <v>85.365853658536579</v>
+      </c>
+      <c r="C36" s="23">
+        <f t="shared" si="4"/>
+        <v>6.833333333333333</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="B37" s="26">
+        <f t="shared" si="3"/>
+        <v>91.428571428571431</v>
+      </c>
+      <c r="C37" s="23">
+        <f t="shared" si="4"/>
+        <v>11.666666666666666</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="B38" s="26">
+        <f t="shared" si="3"/>
+        <v>82.758620689655174</v>
+      </c>
+      <c r="C38" s="23">
+        <f t="shared" si="4"/>
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A39" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="B39" s="26">
+        <f t="shared" si="3"/>
+        <v>72.727272727272734</v>
+      </c>
+      <c r="C39" s="23">
+        <f t="shared" si="4"/>
+        <v>3.6666666666666665</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A41" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="B41" s="25"/>
+      <c r="C41" s="15">
+        <f>M9</f>
+        <v>30.083333333333332</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A42" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="B42" s="25"/>
+      <c r="C42" s="15">
+        <f>B21</f>
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A43" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="B43" s="25"/>
+      <c r="C43" s="15">
+        <f>C41/C42</f>
+        <v>6.6851851851851851</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="7">
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A42:B42"/>
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A13:M13"/>
+    <mergeCell ref="A23:K23"/>
+    <mergeCell ref="A32:F32"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" sqref="A3:A9 A15:A21" xr:uid="{783A1768-A046-488C-8D4E-08B172586A30}">
       <formula1>#REF!</formula1>
     </dataValidation>
@@ -4239,7 +8521,7 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="20" t="s">
         <v>12</v>
       </c>
       <c r="B2" s="4" t="s">
@@ -4281,7 +8563,7 @@
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="20" t="s">
         <v>13</v>
       </c>
       <c r="B3" s="4" t="s">
@@ -4323,7 +8605,7 @@
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="20" t="s">
         <v>14</v>
       </c>
       <c r="B4" s="4" t="s">
@@ -4365,7 +8647,7 @@
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="20" t="s">
         <v>15</v>
       </c>
       <c r="B5" s="4" t="s">
@@ -4407,7 +8689,7 @@
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="20" t="s">
         <v>17</v>
       </c>
       <c r="B6" s="4" t="s">
@@ -4449,7 +8731,7 @@
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="20" t="s">
         <v>18</v>
       </c>
       <c r="B7" s="4" t="s">
@@ -4516,7 +8798,7 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="A2:A9" xr:uid="{03EFABEC-7D33-4C49-A587-08C09411945E}">
       <formula1>#REF!</formula1>
     </dataValidation>
@@ -4530,7 +8812,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20FE204D-0B67-410C-8EE1-3A5778E8BBBD}">
-  <dimension ref="N3:O5"/>
+  <dimension ref="N3:O4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="14" max="14" width="20.1796875" customWidth="1"/>
@@ -4554,11 +8836,34 @@
         <v>30.083333333333332</v>
       </c>
     </row>
-    <row r="5" spans="14:15" x14ac:dyDescent="0.35">
-      <c r="N5" s="14" t="s">
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEE382B1-D37A-449B-883E-4C62399BE496}">
+  <dimension ref="J1:K2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="10" max="10" width="22.36328125" customWidth="1"/>
+    <col min="11" max="11" width="16.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J1" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="K1" s="13" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J2" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="O5" s="15">
+      <c r="K2" s="15">
         <f>'Tiempos Android'!M9</f>
         <v>7.6428571428571432</v>
       </c>

</xml_diff>